<commit_message>
feat: update dynamic select options and sample list
</commit_message>
<xml_diff>
--- a/sample-list.xlsx
+++ b/sample-list.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.14.76\Lens Design\11. 문서\생산납기\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77865846-3A7E-43E4-A361-47DA9377C6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20130" windowHeight="10815"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="190">
   <si>
     <t>국가</t>
   </si>
@@ -562,17 +561,191 @@
   </si>
   <si>
     <t>제안렌즈</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>일본</t>
+  </si>
+  <si>
+    <t>PIA</t>
+  </si>
+  <si>
+    <t>남상규</t>
+  </si>
+  <si>
+    <t>Silver Wolf</t>
+  </si>
+  <si>
+    <t>정세희</t>
+  </si>
+  <si>
+    <t>Charmy Cat</t>
+  </si>
+  <si>
+    <t>국내</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>렌즈미</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>김우현</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>M</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>포멜로 브라운</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>포멜로 그레이</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>포멜로 틸그레이</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>칼립소 BE</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>칼립소 CH</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>칼립소 GR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>키비 코지블랙</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">키비 블랙 </t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">키비 초코 </t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1D -0.75</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1D -1.75</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1D -3.00</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1D -3.50</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1D -3.75</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1D -4.00</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1D -4.50</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1D -5.50</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1D -5.75</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1M -0.75</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1M -1.75</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1M -3.00</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1M -3.50</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1M -3.75</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1M -4.00</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1M -4.50</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1M -5.50</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> Winsome Brown 1M -5.75</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>중동</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Menicon</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>이상윤</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1D</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LIMIMOON 헤이즈 초코</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LIMIMOON 미스트 그레이</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gleam Edge 볼드 브라운</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gleam Edge 볼드 그레이</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.0_ "/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -598,6 +771,14 @@
       <sz val="11"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -648,7 +829,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -680,11 +861,36 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -698,7 +904,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Sheet2"/>
@@ -994,8 +1200,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB42"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AB75"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.25" style="2" customWidth="1"/>
@@ -2507,6 +2713,9 @@
       <c r="Y20" s="2" t="s">
         <v>67</v>
       </c>
+      <c r="Z20" s="4">
+        <v>46092</v>
+      </c>
       <c r="AB20" s="2" t="s">
         <v>97</v>
       </c>
@@ -3102,6 +3311,9 @@
       <c r="X29" s="2" t="s">
         <v>53</v>
       </c>
+      <c r="Y29" s="2" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
@@ -3782,6 +3994,21 @@
       <c r="O39" s="4">
         <v>46078</v>
       </c>
+      <c r="P39" s="4">
+        <v>46084</v>
+      </c>
+      <c r="Q39" s="4">
+        <v>46089</v>
+      </c>
+      <c r="R39" s="4">
+        <v>46090</v>
+      </c>
+      <c r="S39" s="4">
+        <v>46092</v>
+      </c>
+      <c r="T39" s="4">
+        <v>46092</v>
+      </c>
       <c r="V39" s="2" t="s">
         <v>134</v>
       </c>
@@ -3792,7 +4019,7 @@
         <v>100</v>
       </c>
       <c r="Y39" s="2" t="s">
-        <v>58</v>
+        <v>33</v>
       </c>
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.3">
@@ -3956,6 +4183,12 @@
       <c r="P42" s="4">
         <v>46079</v>
       </c>
+      <c r="Q42" s="4">
+        <v>46086</v>
+      </c>
+      <c r="R42" s="4">
+        <v>46087</v>
+      </c>
       <c r="V42" s="2" t="s">
         <v>66</v>
       </c>
@@ -3969,67 +4202,1454 @@
         <v>143</v>
       </c>
     </row>
+    <row r="43" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F43" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G43" s="7">
+        <v>15</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="J43" s="2">
+        <v>1</v>
+      </c>
+      <c r="K43" s="2">
+        <v>2</v>
+      </c>
+      <c r="L43" s="4">
+        <v>46055</v>
+      </c>
+      <c r="M43" s="4">
+        <v>46085</v>
+      </c>
+      <c r="N43" s="6"/>
+      <c r="O43" s="6"/>
+      <c r="P43" s="4">
+        <v>46085</v>
+      </c>
+      <c r="Q43" s="4">
+        <v>46093</v>
+      </c>
+      <c r="R43" s="4">
+        <v>46094</v>
+      </c>
+      <c r="S43" s="4">
+        <v>46094</v>
+      </c>
+      <c r="T43" s="4">
+        <v>46094</v>
+      </c>
+      <c r="V43" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="W43" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X43" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y43" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="44" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F44" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G44" s="7">
+        <v>15</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="J44" s="2">
+        <v>1</v>
+      </c>
+      <c r="K44" s="2">
+        <v>2</v>
+      </c>
+      <c r="L44" s="4">
+        <v>46055</v>
+      </c>
+      <c r="M44" s="4">
+        <v>46085</v>
+      </c>
+      <c r="N44" s="6"/>
+      <c r="O44" s="6"/>
+      <c r="P44" s="4">
+        <v>46085</v>
+      </c>
+      <c r="Q44" s="4">
+        <v>46093</v>
+      </c>
+      <c r="R44" s="4">
+        <v>46094</v>
+      </c>
+      <c r="S44" s="4">
+        <v>46094</v>
+      </c>
+      <c r="T44" s="4">
+        <v>46094</v>
+      </c>
+      <c r="V44" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="W44" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X44" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y44" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="45" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F45" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="G45" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="J45" s="2">
+        <v>1</v>
+      </c>
+      <c r="K45" s="2">
+        <v>1</v>
+      </c>
+      <c r="L45" s="4">
+        <v>46090</v>
+      </c>
+      <c r="N45" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P45" s="4">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="46" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F46" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="G46" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="J46" s="2">
+        <v>1</v>
+      </c>
+      <c r="K46" s="2">
+        <v>1</v>
+      </c>
+      <c r="L46" s="4">
+        <v>46090</v>
+      </c>
+      <c r="N46" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P46" s="4">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="47" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F47" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="G47" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="J47" s="2">
+        <v>1</v>
+      </c>
+      <c r="K47" s="2">
+        <v>1</v>
+      </c>
+      <c r="L47" s="4">
+        <v>46090</v>
+      </c>
+      <c r="N47" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P47" s="4">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="48" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F48" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="G48" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="J48" s="2">
+        <v>1</v>
+      </c>
+      <c r="K48" s="2">
+        <v>1</v>
+      </c>
+      <c r="L48" s="4">
+        <v>46090</v>
+      </c>
+      <c r="N48" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P48" s="4">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F49" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="G49" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="J49" s="2">
+        <v>1</v>
+      </c>
+      <c r="K49" s="2">
+        <v>1</v>
+      </c>
+      <c r="L49" s="4">
+        <v>46090</v>
+      </c>
+      <c r="N49" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P49" s="4">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F50" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="G50" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="J50" s="2">
+        <v>1</v>
+      </c>
+      <c r="K50" s="2">
+        <v>1</v>
+      </c>
+      <c r="L50" s="4">
+        <v>46090</v>
+      </c>
+      <c r="N50" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P50" s="4">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F51" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="G51" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I51" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="J51" s="2">
+        <v>1</v>
+      </c>
+      <c r="K51" s="2">
+        <v>1</v>
+      </c>
+      <c r="L51" s="4">
+        <v>46090</v>
+      </c>
+      <c r="N51" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P51" s="4">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F52" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="G52" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I52" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="J52" s="2">
+        <v>1</v>
+      </c>
+      <c r="K52" s="2">
+        <v>1</v>
+      </c>
+      <c r="L52" s="4">
+        <v>46090</v>
+      </c>
+      <c r="N52" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P52" s="4">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F53" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="G53" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I53" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="J53" s="2">
+        <v>1</v>
+      </c>
+      <c r="K53" s="2">
+        <v>1</v>
+      </c>
+      <c r="L53" s="4">
+        <v>46090</v>
+      </c>
+      <c r="N53" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P53" s="4">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F54" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G54" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I54" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="J54" s="2">
+        <v>1</v>
+      </c>
+      <c r="K54" s="2">
+        <v>1</v>
+      </c>
+      <c r="L54" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F55" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G55" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I55" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="J55" s="2">
+        <v>1</v>
+      </c>
+      <c r="K55" s="2">
+        <v>1</v>
+      </c>
+      <c r="L55" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A56" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F56" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G56" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I56" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="J56" s="2">
+        <v>1</v>
+      </c>
+      <c r="K56" s="2">
+        <v>1</v>
+      </c>
+      <c r="L56" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F57" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G57" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I57" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="J57" s="2">
+        <v>1</v>
+      </c>
+      <c r="K57" s="2">
+        <v>1</v>
+      </c>
+      <c r="L57" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F58" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G58" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I58" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="J58" s="2">
+        <v>1</v>
+      </c>
+      <c r="K58" s="2">
+        <v>1</v>
+      </c>
+      <c r="L58" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F59" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G59" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I59" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="J59" s="2">
+        <v>1</v>
+      </c>
+      <c r="K59" s="2">
+        <v>1</v>
+      </c>
+      <c r="L59" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F60" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G60" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I60" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="J60" s="2">
+        <v>1</v>
+      </c>
+      <c r="K60" s="2">
+        <v>1</v>
+      </c>
+      <c r="L60" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A61" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F61" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G61" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I61" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="J61" s="2">
+        <v>1</v>
+      </c>
+      <c r="K61" s="2">
+        <v>1</v>
+      </c>
+      <c r="L61" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F62" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G62" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I62" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="J62" s="2">
+        <v>1</v>
+      </c>
+      <c r="K62" s="2">
+        <v>1</v>
+      </c>
+      <c r="L62" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F63" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G63" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I63" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="J63" s="2">
+        <v>1</v>
+      </c>
+      <c r="K63" s="2">
+        <v>1</v>
+      </c>
+      <c r="L63" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A64" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F64" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G64" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I64" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="J64" s="2">
+        <v>1</v>
+      </c>
+      <c r="K64" s="2">
+        <v>1</v>
+      </c>
+      <c r="L64" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A65" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F65" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G65" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I65" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="J65" s="2">
+        <v>1</v>
+      </c>
+      <c r="K65" s="2">
+        <v>1</v>
+      </c>
+      <c r="L65" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A66" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F66" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G66" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I66" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="J66" s="2">
+        <v>1</v>
+      </c>
+      <c r="K66" s="2">
+        <v>1</v>
+      </c>
+      <c r="L66" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F67" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G67" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I67" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="J67" s="2">
+        <v>1</v>
+      </c>
+      <c r="K67" s="2">
+        <v>1</v>
+      </c>
+      <c r="L67" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F68" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G68" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I68" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="J68" s="2">
+        <v>1</v>
+      </c>
+      <c r="K68" s="2">
+        <v>1</v>
+      </c>
+      <c r="L68" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A69" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F69" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G69" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I69" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="J69" s="2">
+        <v>1</v>
+      </c>
+      <c r="K69" s="2">
+        <v>1</v>
+      </c>
+      <c r="L69" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A70" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F70" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G70" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I70" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="J70" s="2">
+        <v>1</v>
+      </c>
+      <c r="K70" s="2">
+        <v>1</v>
+      </c>
+      <c r="L70" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F71" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G71" s="7">
+        <v>14.2</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I71" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="J71" s="2">
+        <v>1</v>
+      </c>
+      <c r="K71" s="2">
+        <v>1</v>
+      </c>
+      <c r="L71" s="4">
+        <v>46086</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F72" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G72" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="J72" s="2">
+        <v>1</v>
+      </c>
+      <c r="K72" s="2">
+        <v>1</v>
+      </c>
+      <c r="L72" s="4">
+        <v>46092</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F73" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G73" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="J73" s="2">
+        <v>1</v>
+      </c>
+      <c r="K73" s="2">
+        <v>1</v>
+      </c>
+      <c r="L73" s="4">
+        <v>46092</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F74" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G74" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I74" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="J74" s="2">
+        <v>1</v>
+      </c>
+      <c r="K74" s="2">
+        <v>1</v>
+      </c>
+      <c r="L74" s="4">
+        <v>46092</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A75" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F75" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G75" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H75" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I75" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="J75" s="2">
+        <v>1</v>
+      </c>
+      <c r="K75" s="2">
+        <v>1</v>
+      </c>
+      <c r="L75" s="4">
+        <v>46092</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="V1:V38" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="V1:V38"/>
   <phoneticPr fontId="2" type="noConversion"/>
+  <conditionalFormatting sqref="I51:I53">
+    <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
+      <formula>$E3099:$E1048568="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I62 I71">
+    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
+      <formula>$E3102:$E1048571="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I54:I61 I63:I70">
+    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
+      <formula>$E3095:$E1048564="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="9">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$F$2:$F$4</xm:f>
           </x14:formula1>
-          <xm:sqref>W2:W37 W39:W1048576</xm:sqref>
+          <xm:sqref>W2:W37 Y39 W39:W1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$G$2:$G$5</xm:f>
           </x14:formula1>
           <xm:sqref>X2:X37 X39:X1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$E$2:$E$4</xm:f>
           </x14:formula1>
           <xm:sqref>H2:H37 H39:H1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000003000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$D$2:$D$5</xm:f>
           </x14:formula1>
           <xm:sqref>G2:G37 G39:G1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000004000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$C$2:$C$5</xm:f>
           </x14:formula1>
           <xm:sqref>F2:F37 F39:F1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000005000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$B$2:$B$3</xm:f>
           </x14:formula1>
           <xm:sqref>E2:E37 E39:E1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000006000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$A$2:$A$4</xm:f>
           </x14:formula1>
           <xm:sqref>D2:D37 D39:D1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000008000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>'[복사본 sample-list.xlsx]Sheet2'!#REF!</xm:f>
           </x14:formula1>
           <xm:sqref>D38:H38 W38:X38</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5AA6FBA5-1020-4249-B16C-255F826E1A33}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$H$2:$H$7</xm:f>
           </x14:formula1>
-          <xm:sqref>Y2:Y1048576</xm:sqref>
+          <xm:sqref>Y2:Y38 Y40:Y1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4038,7 +5658,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
chore: update sample list
</commit_message>
<xml_diff>
--- a/sample-list.xlsx
+++ b/sample-list.xlsx
@@ -19,14 +19,14 @@
     <externalReference r:id="rId3"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$V$1:$V$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$V$1:$V$41</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="194">
   <si>
     <t>국가</t>
   </si>
@@ -735,6 +735,22 @@
   </si>
   <si>
     <t>Gleam Edge 볼드 그레이</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SY9-Aurora B</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SY10-C 5th</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>파우더</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SY2</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1201,7 +1217,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB75"/>
+  <dimension ref="A1:AB78"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.25" style="2" customWidth="1"/>
@@ -2675,7 +2691,7 @@
         <v>10</v>
       </c>
       <c r="L20" s="4">
-        <v>45621</v>
+        <v>45644</v>
       </c>
       <c r="M20" s="10">
         <v>46063</v>
@@ -2712,9 +2728,6 @@
       </c>
       <c r="Y20" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="Z20" s="4">
-        <v>46092</v>
       </c>
       <c r="AB20" s="2" t="s">
         <v>97</v>
@@ -2755,7 +2768,7 @@
         <v>10</v>
       </c>
       <c r="L21" s="4">
-        <v>45621</v>
+        <v>45644</v>
       </c>
       <c r="M21" s="10">
         <v>46063</v>
@@ -2792,6 +2805,9 @@
       </c>
       <c r="Y21" s="2" t="s">
         <v>67</v>
+      </c>
+      <c r="Z21" s="4">
+        <v>46092</v>
       </c>
       <c r="AB21" s="2" t="s">
         <v>97</v>
@@ -2823,41 +2839,55 @@
         <v>28</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>107</v>
+        <v>190</v>
       </c>
       <c r="J22" s="2">
         <v>1</v>
       </c>
       <c r="K22" s="2">
-        <v>1</v>
-      </c>
-      <c r="L22" s="6"/>
-      <c r="M22" s="6"/>
-      <c r="N22" s="6"/>
-      <c r="O22" s="6"/>
-      <c r="P22" s="10">
-        <v>46065</v>
-      </c>
-      <c r="Q22" s="10">
-        <v>46075</v>
+        <v>7</v>
+      </c>
+      <c r="L22" s="4">
+        <v>45644</v>
+      </c>
+      <c r="M22" s="10">
+        <v>46063</v>
+      </c>
+      <c r="N22" s="10">
+        <v>45940</v>
+      </c>
+      <c r="O22" s="10">
+        <v>45940</v>
+      </c>
+      <c r="P22" s="4">
+        <v>45959</v>
+      </c>
+      <c r="Q22" s="4">
+        <v>45963</v>
       </c>
       <c r="R22" s="4">
-        <v>46076</v>
+        <v>45965</v>
       </c>
       <c r="S22" s="4">
-        <v>46077</v>
+        <v>45966</v>
       </c>
       <c r="T22" s="4">
-        <v>46077</v>
+        <v>45966</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>76</v>
+        <v>51</v>
       </c>
       <c r="W22" s="2" t="s">
-        <v>29</v>
+        <v>92</v>
       </c>
       <c r="X22" s="2" t="s">
         <v>53</v>
+      </c>
+      <c r="Y22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z22" s="4">
+        <v>46065</v>
       </c>
     </row>
     <row r="23" spans="1:28" x14ac:dyDescent="0.3">
@@ -2886,41 +2916,55 @@
         <v>28</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>108</v>
+        <v>191</v>
       </c>
       <c r="J23" s="2">
         <v>1</v>
       </c>
       <c r="K23" s="2">
-        <v>1</v>
-      </c>
-      <c r="L23" s="6"/>
-      <c r="M23" s="6"/>
-      <c r="N23" s="6"/>
-      <c r="O23" s="6"/>
+        <v>5</v>
+      </c>
+      <c r="L23" s="4">
+        <v>45800</v>
+      </c>
+      <c r="M23" s="10">
+        <v>45999</v>
+      </c>
+      <c r="N23" s="10">
+        <v>46000</v>
+      </c>
+      <c r="O23" s="10">
+        <v>46001</v>
+      </c>
       <c r="P23" s="10">
-        <v>46065</v>
-      </c>
-      <c r="Q23" s="10">
-        <v>46075</v>
+        <v>46011</v>
+      </c>
+      <c r="Q23" s="4">
+        <v>46025</v>
       </c>
       <c r="R23" s="4">
-        <v>46076</v>
+        <v>46034</v>
       </c>
       <c r="S23" s="4">
-        <v>46077</v>
+        <v>46035</v>
       </c>
       <c r="T23" s="4">
-        <v>46077</v>
+        <v>46035</v>
       </c>
       <c r="V23" s="2" t="s">
         <v>76</v>
       </c>
       <c r="W23" s="2" t="s">
-        <v>29</v>
+        <v>92</v>
       </c>
       <c r="X23" s="2" t="s">
         <v>53</v>
+      </c>
+      <c r="Y23" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z23" s="4">
+        <v>46065</v>
       </c>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.3">
@@ -2946,44 +2990,58 @@
         <v>14.5</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>28</v>
+        <v>192</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>109</v>
+        <v>193</v>
       </c>
       <c r="J24" s="2">
         <v>1</v>
       </c>
       <c r="K24" s="2">
-        <v>1</v>
-      </c>
-      <c r="L24" s="6"/>
-      <c r="M24" s="6"/>
-      <c r="N24" s="6"/>
-      <c r="O24" s="6"/>
+        <v>2</v>
+      </c>
+      <c r="L24" s="4">
+        <v>45302</v>
+      </c>
+      <c r="M24" s="10">
+        <v>45645</v>
+      </c>
+      <c r="N24" s="10">
+        <v>45652</v>
+      </c>
+      <c r="O24" s="10">
+        <v>45652</v>
+      </c>
       <c r="P24" s="10">
-        <v>46065</v>
+        <v>45670</v>
       </c>
       <c r="Q24" s="10">
-        <v>46075</v>
-      </c>
-      <c r="R24" s="4">
-        <v>46076</v>
+        <v>45672</v>
+      </c>
+      <c r="R24" s="10">
+        <v>45672</v>
       </c>
       <c r="S24" s="4">
-        <v>46077</v>
+        <v>45673</v>
       </c>
       <c r="T24" s="4">
-        <v>46077</v>
+        <v>45673</v>
       </c>
       <c r="V24" s="2" t="s">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="W24" s="2" t="s">
-        <v>29</v>
+        <v>92</v>
       </c>
       <c r="X24" s="2" t="s">
         <v>53</v>
+      </c>
+      <c r="Y24" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z24" s="4">
+        <v>46092</v>
       </c>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.3">
@@ -3012,7 +3070,7 @@
         <v>28</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="J25" s="2">
         <v>1</v>
@@ -3040,7 +3098,7 @@
         <v>46077</v>
       </c>
       <c r="V25" s="2" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="W25" s="2" t="s">
         <v>29</v>
@@ -3069,13 +3127,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G26" s="7">
-        <v>15</v>
+        <v>14.5</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="J26" s="2">
         <v>1</v>
@@ -3132,13 +3190,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G27" s="7">
-        <v>15</v>
+        <v>14.5</v>
       </c>
       <c r="H27" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="J27" s="2">
         <v>1</v>
@@ -3174,9 +3232,6 @@
       <c r="X27" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="Y27" s="2" t="s">
-        <v>58</v>
-      </c>
     </row>
     <row r="28" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
@@ -3198,13 +3253,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G28" s="7">
-        <v>15</v>
+        <v>14.5</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="J28" s="2">
         <v>1</v>
@@ -3217,13 +3272,13 @@
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
       <c r="P28" s="10">
-        <v>46066</v>
+        <v>46065</v>
       </c>
       <c r="Q28" s="10">
-        <v>46071</v>
+        <v>46075</v>
       </c>
       <c r="R28" s="4">
-        <v>46077</v>
+        <v>46076</v>
       </c>
       <c r="S28" s="4">
         <v>46077</v>
@@ -3243,13 +3298,13 @@
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>34</v>
@@ -3261,13 +3316,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G29" s="7">
-        <v>14.5</v>
+        <v>15</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="J29" s="2">
         <v>1</v>
@@ -3275,55 +3330,44 @@
       <c r="K29" s="2">
         <v>1</v>
       </c>
-      <c r="L29" s="10">
-        <v>46063</v>
-      </c>
-      <c r="M29" s="10">
-        <v>46063</v>
-      </c>
-      <c r="N29" s="10">
-        <v>46063</v>
-      </c>
-      <c r="O29" s="10">
-        <v>46066</v>
-      </c>
+      <c r="L29" s="6"/>
+      <c r="M29" s="6"/>
+      <c r="N29" s="6"/>
+      <c r="O29" s="6"/>
       <c r="P29" s="10">
-        <v>46074</v>
-      </c>
-      <c r="Q29" s="4">
+        <v>46065</v>
+      </c>
+      <c r="Q29" s="10">
+        <v>46075</v>
+      </c>
+      <c r="R29" s="4">
         <v>46076</v>
       </c>
-      <c r="R29" s="4">
-        <v>46078</v>
-      </c>
       <c r="S29" s="4">
-        <v>46080</v>
+        <v>46077</v>
       </c>
       <c r="T29" s="4">
-        <v>46080</v>
+        <v>46077</v>
       </c>
       <c r="V29" s="2" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="W29" s="2" t="s">
-        <v>96</v>
+        <v>29</v>
       </c>
       <c r="X29" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="Y29" s="2" t="s">
-        <v>58</v>
-      </c>
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>34</v>
@@ -3341,7 +3385,7 @@
         <v>28</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="J30" s="2">
         <v>1</v>
@@ -3349,32 +3393,30 @@
       <c r="K30" s="2">
         <v>1</v>
       </c>
-      <c r="L30" s="4">
-        <v>46052</v>
-      </c>
+      <c r="L30" s="6"/>
       <c r="M30" s="6"/>
       <c r="N30" s="6"/>
       <c r="O30" s="6"/>
-      <c r="P30" s="4">
-        <v>46053</v>
-      </c>
-      <c r="Q30" s="4">
+      <c r="P30" s="10">
         <v>46065</v>
       </c>
+      <c r="Q30" s="10">
+        <v>46075</v>
+      </c>
       <c r="R30" s="4">
-        <v>46066</v>
+        <v>46076</v>
       </c>
       <c r="S30" s="4">
-        <v>46066</v>
+        <v>46077</v>
       </c>
       <c r="T30" s="4">
-        <v>46066</v>
+        <v>46077</v>
       </c>
       <c r="V30" s="2" t="s">
-        <v>123</v>
+        <v>98</v>
       </c>
       <c r="W30" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="X30" s="2" t="s">
         <v>53</v>
@@ -3385,13 +3427,13 @@
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>34</v>
@@ -3409,7 +3451,7 @@
         <v>28</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="J31" s="2">
         <v>1</v>
@@ -3417,49 +3459,44 @@
       <c r="K31" s="2">
         <v>1</v>
       </c>
-      <c r="L31" s="4">
-        <v>46052</v>
-      </c>
+      <c r="L31" s="6"/>
       <c r="M31" s="6"/>
       <c r="N31" s="6"/>
       <c r="O31" s="6"/>
-      <c r="P31" s="4">
-        <v>46053</v>
-      </c>
-      <c r="Q31" s="4">
-        <v>46065</v>
+      <c r="P31" s="10">
+        <v>46066</v>
+      </c>
+      <c r="Q31" s="10">
+        <v>46071</v>
       </c>
       <c r="R31" s="4">
-        <v>46066</v>
+        <v>46077</v>
       </c>
       <c r="S31" s="4">
-        <v>46066</v>
+        <v>46077</v>
       </c>
       <c r="T31" s="4">
-        <v>46066</v>
+        <v>46077</v>
       </c>
       <c r="V31" s="2" t="s">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="W31" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="X31" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="Y31" s="2" t="s">
-        <v>58</v>
-      </c>
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>106</v>
+        <v>43</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>105</v>
+        <v>44</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>34</v>
@@ -3471,13 +3508,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G32" s="7">
-        <v>15</v>
+        <v>14.5</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="J32" s="2">
         <v>1</v>
@@ -3485,32 +3522,38 @@
       <c r="K32" s="2">
         <v>1</v>
       </c>
-      <c r="L32" s="4">
-        <v>46052</v>
-      </c>
-      <c r="M32" s="6"/>
-      <c r="N32" s="6"/>
-      <c r="O32" s="6"/>
-      <c r="P32" s="4">
-        <v>46053</v>
+      <c r="L32" s="10">
+        <v>46063</v>
+      </c>
+      <c r="M32" s="10">
+        <v>46063</v>
+      </c>
+      <c r="N32" s="10">
+        <v>46063</v>
+      </c>
+      <c r="O32" s="10">
+        <v>46066</v>
+      </c>
+      <c r="P32" s="10">
+        <v>46074</v>
       </c>
       <c r="Q32" s="4">
-        <v>46065</v>
+        <v>46076</v>
       </c>
       <c r="R32" s="4">
-        <v>46066</v>
+        <v>46078</v>
       </c>
       <c r="S32" s="4">
-        <v>46066</v>
+        <v>46080</v>
       </c>
       <c r="T32" s="4">
-        <v>46066</v>
+        <v>46080</v>
       </c>
       <c r="V32" s="2" t="s">
-        <v>123</v>
+        <v>94</v>
       </c>
       <c r="W32" s="2" t="s">
-        <v>30</v>
+        <v>96</v>
       </c>
       <c r="X32" s="2" t="s">
         <v>53</v>
@@ -3521,13 +3564,13 @@
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>34</v>
@@ -3539,34 +3582,28 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G33" s="7">
-        <v>14.5</v>
+        <v>15</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>136</v>
+        <v>101</v>
       </c>
       <c r="J33" s="2">
         <v>1</v>
       </c>
       <c r="K33" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L33" s="4">
-        <v>45868</v>
-      </c>
-      <c r="M33" s="4">
-        <v>46055</v>
-      </c>
-      <c r="N33" s="4">
-        <v>46056</v>
-      </c>
-      <c r="O33" s="4">
-        <v>46056</v>
-      </c>
+        <v>46052</v>
+      </c>
+      <c r="M33" s="6"/>
+      <c r="N33" s="6"/>
+      <c r="O33" s="6"/>
       <c r="P33" s="4">
-        <v>46058</v>
+        <v>46053</v>
       </c>
       <c r="Q33" s="4">
         <v>46065</v>
@@ -3581,24 +3618,27 @@
         <v>46066</v>
       </c>
       <c r="V33" s="2" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="W33" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X33" s="2" t="s">
         <v>53</v>
       </c>
+      <c r="Y33" s="2" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>34</v>
@@ -3610,34 +3650,28 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G34" s="7">
-        <v>14.5</v>
+        <v>15</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="J34" s="2">
         <v>1</v>
       </c>
       <c r="K34" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L34" s="4">
-        <v>45868</v>
-      </c>
-      <c r="M34" s="4">
-        <v>46055</v>
-      </c>
-      <c r="N34" s="4">
-        <v>46056</v>
-      </c>
-      <c r="O34" s="4">
-        <v>46056</v>
-      </c>
+        <v>46052</v>
+      </c>
+      <c r="M34" s="6"/>
+      <c r="N34" s="6"/>
+      <c r="O34" s="6"/>
       <c r="P34" s="4">
-        <v>46058</v>
+        <v>46053</v>
       </c>
       <c r="Q34" s="4">
         <v>46065</v>
@@ -3652,24 +3686,27 @@
         <v>46066</v>
       </c>
       <c r="V34" s="2" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="W34" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X34" s="2" t="s">
         <v>53</v>
       </c>
+      <c r="Y34" s="2" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>34</v>
@@ -3681,34 +3718,28 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G35" s="7">
-        <v>14.5</v>
+        <v>15</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="J35" s="2">
         <v>1</v>
       </c>
       <c r="K35" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L35" s="4">
-        <v>45868</v>
-      </c>
-      <c r="M35" s="4">
-        <v>46055</v>
-      </c>
-      <c r="N35" s="4">
-        <v>46056</v>
-      </c>
-      <c r="O35" s="4">
-        <v>46056</v>
-      </c>
+        <v>46052</v>
+      </c>
+      <c r="M35" s="6"/>
+      <c r="N35" s="6"/>
+      <c r="O35" s="6"/>
       <c r="P35" s="4">
-        <v>46057</v>
+        <v>46053</v>
       </c>
       <c r="Q35" s="4">
         <v>46065</v>
@@ -3723,13 +3754,16 @@
         <v>46066</v>
       </c>
       <c r="V35" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="W35" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X35" s="2" t="s">
         <v>53</v>
+      </c>
+      <c r="Y35" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.3">
@@ -3758,7 +3792,7 @@
         <v>28</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="J36" s="2">
         <v>1</v>
@@ -3794,7 +3828,7 @@
         <v>46066</v>
       </c>
       <c r="V36" s="2" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="W36" s="2" t="s">
         <v>29</v>
@@ -3829,7 +3863,7 @@
         <v>28</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="J37" s="2">
         <v>1</v>
@@ -3865,7 +3899,7 @@
         <v>46066</v>
       </c>
       <c r="V37" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="W37" s="2" t="s">
         <v>29</v>
@@ -3876,52 +3910,52 @@
     </row>
     <row r="38" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="F38" s="3">
         <v>0.55000000000000004</v>
       </c>
       <c r="G38" s="7">
-        <v>14.2</v>
+        <v>14.5</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="J38" s="2">
         <v>1</v>
       </c>
       <c r="K38" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L38" s="4">
-        <v>46062</v>
+        <v>45868</v>
       </c>
       <c r="M38" s="4">
-        <v>46062</v>
+        <v>46055</v>
       </c>
       <c r="N38" s="4">
-        <v>46063</v>
+        <v>46056</v>
       </c>
       <c r="O38" s="4">
-        <v>46063</v>
+        <v>46056</v>
       </c>
       <c r="P38" s="4">
-        <v>46063</v>
+        <v>46057</v>
       </c>
       <c r="Q38" s="4">
         <v>46065</v>
@@ -3930,107 +3964,101 @@
         <v>46066</v>
       </c>
       <c r="S38" s="4">
-        <v>46072</v>
+        <v>46066</v>
       </c>
       <c r="T38" s="4">
-        <v>46072</v>
+        <v>46066</v>
       </c>
       <c r="V38" s="2" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="W38" s="2" t="s">
-        <v>131</v>
+        <v>29</v>
       </c>
       <c r="X38" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="Y38" s="2" t="s">
-        <v>58</v>
-      </c>
     </row>
     <row r="39" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>43</v>
+        <v>116</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>44</v>
+        <v>115</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>45</v>
+        <v>114</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="F39" s="3">
-        <v>0.43</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="G39" s="7">
-        <v>14.2</v>
+        <v>14.5</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>132</v>
+        <v>28</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="J39" s="2">
         <v>1</v>
       </c>
       <c r="K39" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L39" s="4">
-        <v>46077</v>
+        <v>45868</v>
       </c>
       <c r="M39" s="4">
-        <v>46077</v>
+        <v>46055</v>
       </c>
       <c r="N39" s="4">
-        <v>46078</v>
+        <v>46056</v>
       </c>
       <c r="O39" s="4">
-        <v>46078</v>
+        <v>46056</v>
       </c>
       <c r="P39" s="4">
-        <v>46084</v>
+        <v>46058</v>
       </c>
       <c r="Q39" s="4">
-        <v>46089</v>
+        <v>46065</v>
       </c>
       <c r="R39" s="4">
-        <v>46090</v>
+        <v>46066</v>
       </c>
       <c r="S39" s="4">
-        <v>46092</v>
+        <v>46066</v>
       </c>
       <c r="T39" s="4">
-        <v>46092</v>
+        <v>46066</v>
       </c>
       <c r="V39" s="2" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="W39" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="X39" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="Y39" s="2" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>62</v>
+        <v>116</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>63</v>
+        <v>115</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>64</v>
+        <v>114</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>34</v>
@@ -4048,66 +4076,78 @@
         <v>28</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="J40" s="2">
         <v>1</v>
       </c>
       <c r="K40" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L40" s="4">
+        <v>45868</v>
+      </c>
+      <c r="M40" s="4">
+        <v>46055</v>
+      </c>
+      <c r="N40" s="4">
+        <v>46056</v>
+      </c>
+      <c r="O40" s="4">
+        <v>46056</v>
+      </c>
+      <c r="P40" s="4">
+        <v>46058</v>
+      </c>
+      <c r="Q40" s="4">
+        <v>46065</v>
+      </c>
+      <c r="R40" s="4">
         <v>46066</v>
       </c>
-      <c r="M40" s="6"/>
-      <c r="N40" s="6"/>
-      <c r="O40" s="6"/>
-      <c r="P40" s="4">
-        <v>46076</v>
-      </c>
-      <c r="Q40" s="4">
-        <v>46083</v>
+      <c r="S40" s="4">
+        <v>46066</v>
+      </c>
+      <c r="T40" s="4">
+        <v>46066</v>
       </c>
       <c r="V40" s="2" t="s">
-        <v>52</v>
+        <v>118</v>
       </c>
       <c r="W40" s="2" t="s">
         <v>29</v>
       </c>
       <c r="X40" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="Y40" s="2" t="s">
-        <v>143</v>
+        <v>53</v>
       </c>
     </row>
     <row r="41" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>62</v>
+        <v>126</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>63</v>
+        <v>127</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F41" s="3">
         <v>0.55000000000000004</v>
       </c>
       <c r="G41" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="J41" s="2">
         <v>1</v>
@@ -4116,57 +4156,72 @@
         <v>1</v>
       </c>
       <c r="L41" s="4">
+        <v>46062</v>
+      </c>
+      <c r="M41" s="4">
+        <v>46062</v>
+      </c>
+      <c r="N41" s="4">
+        <v>46063</v>
+      </c>
+      <c r="O41" s="4">
+        <v>46063</v>
+      </c>
+      <c r="P41" s="4">
+        <v>46063</v>
+      </c>
+      <c r="Q41" s="4">
+        <v>46065</v>
+      </c>
+      <c r="R41" s="4">
         <v>46066</v>
       </c>
-      <c r="M41" s="6"/>
-      <c r="N41" s="6"/>
-      <c r="O41" s="6"/>
-      <c r="P41" s="4">
-        <v>46076</v>
-      </c>
-      <c r="Q41" s="4">
-        <v>46083</v>
+      <c r="S41" s="4">
+        <v>46072</v>
+      </c>
+      <c r="T41" s="4">
+        <v>46072</v>
       </c>
       <c r="V41" s="2" t="s">
-        <v>52</v>
+        <v>130</v>
       </c>
       <c r="W41" s="2" t="s">
-        <v>29</v>
+        <v>131</v>
       </c>
       <c r="X41" s="2" t="s">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="Y41" s="2" t="s">
-        <v>143</v>
+        <v>58</v>
       </c>
     </row>
     <row r="42" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F42" s="3">
-        <v>0.55000000000000004</v>
+        <v>0.43</v>
       </c>
       <c r="G42" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>28</v>
+        <v>132</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="J42" s="2">
         <v>1</v>
@@ -4175,42 +4230,54 @@
         <v>1</v>
       </c>
       <c r="L42" s="4">
-        <v>46066</v>
-      </c>
-      <c r="M42" s="6"/>
-      <c r="N42" s="6"/>
-      <c r="O42" s="6"/>
+        <v>46077</v>
+      </c>
+      <c r="M42" s="4">
+        <v>46077</v>
+      </c>
+      <c r="N42" s="4">
+        <v>46078</v>
+      </c>
+      <c r="O42" s="4">
+        <v>46078</v>
+      </c>
       <c r="P42" s="4">
-        <v>46079</v>
+        <v>46084</v>
       </c>
       <c r="Q42" s="4">
-        <v>46086</v>
+        <v>46089</v>
       </c>
       <c r="R42" s="4">
-        <v>46087</v>
+        <v>46090</v>
+      </c>
+      <c r="S42" s="4">
+        <v>46092</v>
+      </c>
+      <c r="T42" s="4">
+        <v>46092</v>
       </c>
       <c r="V42" s="2" t="s">
-        <v>66</v>
+        <v>134</v>
       </c>
       <c r="W42" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="X42" s="2" t="s">
         <v>100</v>
       </c>
       <c r="Y42" s="2" t="s">
-        <v>143</v>
+        <v>33</v>
       </c>
     </row>
     <row r="43" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>145</v>
+        <v>62</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>146</v>
+        <v>63</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>147</v>
+        <v>64</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>34</v>
@@ -4222,48 +4289,37 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G43" s="7">
-        <v>15</v>
+        <v>14.5</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="J43" s="2">
         <v>1</v>
       </c>
       <c r="K43" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L43" s="4">
-        <v>46055</v>
-      </c>
-      <c r="M43" s="4">
-        <v>46085</v>
-      </c>
+        <v>46066</v>
+      </c>
+      <c r="M43" s="6"/>
       <c r="N43" s="6"/>
       <c r="O43" s="6"/>
       <c r="P43" s="4">
-        <v>46085</v>
+        <v>46076</v>
       </c>
       <c r="Q43" s="4">
-        <v>46093</v>
-      </c>
-      <c r="R43" s="4">
-        <v>46094</v>
-      </c>
-      <c r="S43" s="4">
-        <v>46094</v>
-      </c>
-      <c r="T43" s="4">
-        <v>46094</v>
+        <v>46083</v>
       </c>
       <c r="V43" s="2" t="s">
-        <v>149</v>
+        <v>52</v>
       </c>
       <c r="W43" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="X43" s="2" t="s">
         <v>100</v>
@@ -4274,13 +4330,13 @@
     </row>
     <row r="44" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>145</v>
+        <v>62</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>146</v>
+        <v>63</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>147</v>
+        <v>64</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>34</v>
@@ -4292,48 +4348,37 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G44" s="7">
-        <v>15</v>
+        <v>14.5</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="J44" s="2">
         <v>1</v>
       </c>
       <c r="K44" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L44" s="4">
-        <v>46055</v>
-      </c>
-      <c r="M44" s="4">
-        <v>46085</v>
-      </c>
+        <v>46066</v>
+      </c>
+      <c r="M44" s="6"/>
       <c r="N44" s="6"/>
       <c r="O44" s="6"/>
       <c r="P44" s="4">
-        <v>46085</v>
+        <v>46076</v>
       </c>
       <c r="Q44" s="4">
-        <v>46093</v>
-      </c>
-      <c r="R44" s="4">
-        <v>46094</v>
-      </c>
-      <c r="S44" s="4">
-        <v>46094</v>
-      </c>
-      <c r="T44" s="4">
-        <v>46094</v>
+        <v>46083</v>
       </c>
       <c r="V44" s="2" t="s">
-        <v>149</v>
+        <v>52</v>
       </c>
       <c r="W44" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="X44" s="2" t="s">
         <v>100</v>
@@ -4344,31 +4389,31 @@
     </row>
     <row r="45" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>151</v>
+        <v>62</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>152</v>
+        <v>63</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>153</v>
+        <v>64</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>154</v>
+        <v>27</v>
       </c>
       <c r="F45" s="3">
-        <v>0.45</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="G45" s="7">
-        <v>14.2</v>
+        <v>14.5</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="J45" s="2">
         <v>1</v>
@@ -4377,101 +4422,171 @@
         <v>1</v>
       </c>
       <c r="L45" s="4">
-        <v>46090</v>
-      </c>
-      <c r="N45" s="4">
-        <v>46085</v>
-      </c>
+        <v>46066</v>
+      </c>
+      <c r="M45" s="6"/>
+      <c r="N45" s="6"/>
+      <c r="O45" s="6"/>
       <c r="P45" s="4">
+        <v>46079</v>
+      </c>
+      <c r="Q45" s="4">
+        <v>46086</v>
+      </c>
+      <c r="R45" s="4">
         <v>46087</v>
+      </c>
+      <c r="V45" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="W45" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X45" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y45" s="2" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="46" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>154</v>
+        <v>27</v>
       </c>
       <c r="F46" s="3">
-        <v>0.45</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="G46" s="7">
-        <v>14.2</v>
+        <v>15</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="J46" s="2">
         <v>1</v>
       </c>
       <c r="K46" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L46" s="4">
-        <v>46090</v>
-      </c>
-      <c r="N46" s="4">
+        <v>46055</v>
+      </c>
+      <c r="M46" s="4">
         <v>46085</v>
       </c>
+      <c r="N46" s="6"/>
+      <c r="O46" s="6"/>
       <c r="P46" s="4">
-        <v>46087</v>
+        <v>46085</v>
+      </c>
+      <c r="Q46" s="4">
+        <v>46093</v>
+      </c>
+      <c r="R46" s="4">
+        <v>46094</v>
+      </c>
+      <c r="S46" s="4">
+        <v>46094</v>
+      </c>
+      <c r="T46" s="4">
+        <v>46094</v>
+      </c>
+      <c r="V46" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="W46" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X46" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y46" s="2" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="47" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>154</v>
+        <v>27</v>
       </c>
       <c r="F47" s="3">
-        <v>0.45</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="G47" s="7">
-        <v>14.2</v>
+        <v>15</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>28</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="J47" s="2">
         <v>1</v>
       </c>
       <c r="K47" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L47" s="4">
-        <v>46090</v>
-      </c>
-      <c r="N47" s="4">
+        <v>46055</v>
+      </c>
+      <c r="M47" s="4">
         <v>46085</v>
       </c>
+      <c r="N47" s="6"/>
+      <c r="O47" s="6"/>
       <c r="P47" s="4">
-        <v>46087</v>
+        <v>46085</v>
+      </c>
+      <c r="Q47" s="4">
+        <v>46093</v>
+      </c>
+      <c r="R47" s="4">
+        <v>46094</v>
+      </c>
+      <c r="S47" s="4">
+        <v>46094</v>
+      </c>
+      <c r="T47" s="4">
+        <v>46094</v>
+      </c>
+      <c r="V47" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="W47" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X47" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y47" s="2" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="48" spans="1:25" x14ac:dyDescent="0.3">
@@ -4500,7 +4615,7 @@
         <v>28</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="J48" s="2">
         <v>1</v>
@@ -4544,7 +4659,7 @@
         <v>28</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="J49" s="2">
         <v>1</v>
@@ -4588,7 +4703,7 @@
         <v>28</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="J50" s="2">
         <v>1</v>
@@ -4631,8 +4746,8 @@
       <c r="H51" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I51" s="11" t="s">
-        <v>161</v>
+      <c r="I51" s="2" t="s">
+        <v>158</v>
       </c>
       <c r="J51" s="2">
         <v>1</v>
@@ -4675,8 +4790,8 @@
       <c r="H52" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I52" s="11" t="s">
-        <v>162</v>
+      <c r="I52" s="2" t="s">
+        <v>159</v>
       </c>
       <c r="J52" s="2">
         <v>1</v>
@@ -4719,8 +4834,8 @@
       <c r="H53" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I53" s="11" t="s">
-        <v>163</v>
+      <c r="I53" s="2" t="s">
+        <v>160</v>
       </c>
       <c r="J53" s="2">
         <v>1</v>
@@ -4740,22 +4855,22 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>182</v>
+        <v>151</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>183</v>
+        <v>152</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>184</v>
+        <v>153</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>185</v>
+        <v>154</v>
       </c>
       <c r="F54" s="3">
-        <v>0.55000000000000004</v>
+        <v>0.45</v>
       </c>
       <c r="G54" s="7">
         <v>14.2</v>
@@ -4764,7 +4879,7 @@
         <v>28</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="J54" s="2">
         <v>1</v>
@@ -4773,27 +4888,33 @@
         <v>1</v>
       </c>
       <c r="L54" s="4">
-        <v>46086</v>
+        <v>46090</v>
+      </c>
+      <c r="N54" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P54" s="4">
+        <v>46087</v>
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>182</v>
+        <v>151</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>183</v>
+        <v>152</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>184</v>
+        <v>153</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>185</v>
+        <v>154</v>
       </c>
       <c r="F55" s="3">
-        <v>0.55000000000000004</v>
+        <v>0.45</v>
       </c>
       <c r="G55" s="7">
         <v>14.2</v>
@@ -4802,7 +4923,7 @@
         <v>28</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="J55" s="2">
         <v>1</v>
@@ -4811,27 +4932,33 @@
         <v>1</v>
       </c>
       <c r="L55" s="4">
-        <v>46086</v>
+        <v>46090</v>
+      </c>
+      <c r="N55" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P55" s="4">
+        <v>46087</v>
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>182</v>
+        <v>151</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>183</v>
+        <v>152</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>184</v>
+        <v>153</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>26</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>27</v>
+        <v>154</v>
       </c>
       <c r="F56" s="3">
-        <v>0.55000000000000004</v>
+        <v>0.45</v>
       </c>
       <c r="G56" s="7">
         <v>14.2</v>
@@ -4840,7 +4967,7 @@
         <v>28</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="J56" s="2">
         <v>1</v>
@@ -4849,7 +4976,13 @@
         <v>1</v>
       </c>
       <c r="L56" s="4">
-        <v>46086</v>
+        <v>46090</v>
+      </c>
+      <c r="N56" s="4">
+        <v>46085</v>
+      </c>
+      <c r="P56" s="4">
+        <v>46087</v>
       </c>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.3">
@@ -4866,7 +4999,7 @@
         <v>26</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>27</v>
+        <v>185</v>
       </c>
       <c r="F57" s="3">
         <v>0.55000000000000004</v>
@@ -4878,7 +5011,7 @@
         <v>28</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J57" s="2">
         <v>1</v>
@@ -4904,7 +5037,7 @@
         <v>26</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>27</v>
+        <v>185</v>
       </c>
       <c r="F58" s="3">
         <v>0.55000000000000004</v>
@@ -4916,7 +5049,7 @@
         <v>28</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="J58" s="2">
         <v>1</v>
@@ -4954,7 +5087,7 @@
         <v>28</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="J59" s="2">
         <v>1</v>
@@ -4992,7 +5125,7 @@
         <v>28</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="J60" s="2">
         <v>1</v>
@@ -5030,7 +5163,7 @@
         <v>28</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="J61" s="2">
         <v>1</v>
@@ -5068,7 +5201,7 @@
         <v>28</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J62" s="2">
         <v>1</v>
@@ -5106,7 +5239,7 @@
         <v>28</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="J63" s="2">
         <v>1</v>
@@ -5144,7 +5277,7 @@
         <v>28</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J64" s="2">
         <v>1</v>
@@ -5182,7 +5315,7 @@
         <v>28</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="J65" s="2">
         <v>1</v>
@@ -5220,7 +5353,7 @@
         <v>28</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="J66" s="2">
         <v>1</v>
@@ -5258,7 +5391,7 @@
         <v>28</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="J67" s="2">
         <v>1</v>
@@ -5296,7 +5429,7 @@
         <v>28</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="J68" s="2">
         <v>1</v>
@@ -5334,7 +5467,7 @@
         <v>28</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="J69" s="2">
         <v>1</v>
@@ -5372,7 +5505,7 @@
         <v>28</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="J70" s="2">
         <v>1</v>
@@ -5410,7 +5543,7 @@
         <v>28</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="J71" s="2">
         <v>1</v>
@@ -5424,16 +5557,16 @@
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>151</v>
+        <v>182</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>152</v>
+        <v>183</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>153</v>
+        <v>184</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>27</v>
@@ -5442,13 +5575,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G72" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I72" s="2" t="s">
-        <v>186</v>
+      <c r="I72" s="11" t="s">
+        <v>179</v>
       </c>
       <c r="J72" s="2">
         <v>1</v>
@@ -5457,21 +5590,21 @@
         <v>1</v>
       </c>
       <c r="L72" s="4">
-        <v>46092</v>
+        <v>46086</v>
       </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>151</v>
+        <v>182</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>152</v>
+        <v>183</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>153</v>
+        <v>184</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>27</v>
@@ -5480,13 +5613,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G73" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I73" s="2" t="s">
-        <v>187</v>
+      <c r="I73" s="11" t="s">
+        <v>180</v>
       </c>
       <c r="J73" s="2">
         <v>1</v>
@@ -5495,21 +5628,21 @@
         <v>1</v>
       </c>
       <c r="L73" s="4">
-        <v>46092</v>
+        <v>46086</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
-        <v>151</v>
+        <v>182</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>152</v>
+        <v>183</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>153</v>
+        <v>184</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>27</v>
@@ -5518,13 +5651,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G74" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H74" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I74" s="2" t="s">
-        <v>188</v>
+      <c r="I74" s="11" t="s">
+        <v>181</v>
       </c>
       <c r="J74" s="2">
         <v>1</v>
@@ -5533,7 +5666,7 @@
         <v>1</v>
       </c>
       <c r="L74" s="4">
-        <v>46092</v>
+        <v>46086</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.3">
@@ -5562,7 +5695,7 @@
         <v>28</v>
       </c>
       <c r="I75" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="J75" s="2">
         <v>1</v>
@@ -5574,22 +5707,136 @@
         <v>46092</v>
       </c>
     </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F76" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G76" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H76" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I76" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="J76" s="2">
+        <v>1</v>
+      </c>
+      <c r="K76" s="2">
+        <v>1</v>
+      </c>
+      <c r="L76" s="4">
+        <v>46092</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A77" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F77" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G77" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H77" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I77" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="J77" s="2">
+        <v>1</v>
+      </c>
+      <c r="K77" s="2">
+        <v>1</v>
+      </c>
+      <c r="L77" s="4">
+        <v>46092</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A78" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F78" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G78" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H78" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I78" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="J78" s="2">
+        <v>1</v>
+      </c>
+      <c r="K78" s="2">
+        <v>1</v>
+      </c>
+      <c r="L78" s="4">
+        <v>46092</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="V1:V38"/>
+  <autoFilter ref="V1:V41"/>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="I51:I53">
+  <conditionalFormatting sqref="I54:I56">
     <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
-      <formula>$E3099:$E1048568="sub"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I62 I71">
-    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
       <formula>$E3102:$E1048571="sub"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I54:I61 I63:I70">
+  <conditionalFormatting sqref="I65 I74">
+    <cfRule type="expression" dxfId="1" priority="2" stopIfTrue="1">
+      <formula>$E3105:$E1048574="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I57:I64 I66:I73">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
-      <formula>$E3095:$E1048564="sub"</formula>
+      <formula>$E3098:$E1048567="sub"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5601,55 +5848,55 @@
           <x14:formula1>
             <xm:f>Sheet2!$F$2:$F$4</xm:f>
           </x14:formula1>
-          <xm:sqref>W2:W37 Y39 W39:W1048576</xm:sqref>
+          <xm:sqref>W42:W1048576 Y42 W2:W40</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$G$2:$G$5</xm:f>
           </x14:formula1>
-          <xm:sqref>X2:X37 X39:X1048576</xm:sqref>
+          <xm:sqref>X42:X1048576 X2:X40</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$E$2:$E$4</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H37 H39:H1048576</xm:sqref>
+          <xm:sqref>H42:H1048576 H2:H40</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$D$2:$D$5</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:G37 G39:G1048576</xm:sqref>
+          <xm:sqref>G42:G1048576 G2:G40</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$C$2:$C$5</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F37 F39:F1048576</xm:sqref>
+          <xm:sqref>F42:F1048576 F2:F40</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$B$2:$B$3</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E37 E39:E1048576</xm:sqref>
+          <xm:sqref>E42:E1048576 E2:E40</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$A$2:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D37 D39:D1048576</xm:sqref>
+          <xm:sqref>D42:D1048576 D2:D40</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>'[복사본 sample-list.xlsx]Sheet2'!#REF!</xm:f>
           </x14:formula1>
-          <xm:sqref>D38:H38 W38:X38</xm:sqref>
+          <xm:sqref>D41:H41 W41:X41</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$H$2:$H$7</xm:f>
           </x14:formula1>
-          <xm:sqref>Y2:Y38 Y40:Y1048576</xm:sqref>
+          <xm:sqref>Y43:Y1048576 Y2:Y41</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Update sample list data
</commit_message>
<xml_diff>
--- a/sample-list.xlsx
+++ b/sample-list.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1086" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="230">
   <si>
     <t>국가</t>
   </si>
@@ -869,14 +869,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Winsome brown 1M -2.00</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Winsome brown 1M -2.25</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Winsome brown 1M -3.00</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -885,10 +877,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Winsome brown 1M -3.25</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Winsome brown 1M -3.75</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -897,22 +885,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Winsome brown 1M -4.25</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Winsome brown 1M -4.50</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Winsome brown 1M -5.00</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Winsome brown 1M -5.25</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Winsome brown 1M -5.50</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -921,11 +897,65 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Winsome brown 1M -6.00</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Winsome brown 1M -7.50</t>
+    <t>Mystical Black 1D -2.00</t>
+  </si>
+  <si>
+    <t>Mystical Black 1D -2.25</t>
+  </si>
+  <si>
+    <t>Mystical Black 1D -3.25</t>
+  </si>
+  <si>
+    <t>Mystical Black 1D -3.5</t>
+  </si>
+  <si>
+    <t>Mystical Black 1D -4.25</t>
+  </si>
+  <si>
+    <t>Mystical Black 1D -5.00</t>
+  </si>
+  <si>
+    <t>Mystical Black 1D -5.25</t>
+  </si>
+  <si>
+    <t>Mystical Black 1D -6.00</t>
+  </si>
+  <si>
+    <t>Shimmering Gray 1D -2.00</t>
+  </si>
+  <si>
+    <t>Shimmering Gray 1D -2.25</t>
+  </si>
+  <si>
+    <t>Shimmering Gray 1D -3.00</t>
+  </si>
+  <si>
+    <t>Shimmering Gray 1D -3.25</t>
+  </si>
+  <si>
+    <t>Shimmering Gray 1D -3.50</t>
+  </si>
+  <si>
+    <t>Shimmering Gray 1D -4.25</t>
+  </si>
+  <si>
+    <t>Shimmering Gray 1D -5.25</t>
+  </si>
+  <si>
+    <t>Shimmering Gray 1D -7.50</t>
+  </si>
+  <si>
+    <t>류미리</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Brilliant Brown 1M -3.00</t>
+  </si>
+  <si>
+    <t>Misty Grey 1M -3.00</t>
+  </si>
+  <si>
+    <t>임수빈</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1079,7 +1109,84 @@
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="22">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1468,7 +1575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB96"/>
+  <dimension ref="A1:AB106"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.25" style="2" customWidth="1"/>
@@ -4140,6 +4247,15 @@
       <c r="Q37" s="4">
         <v>46100</v>
       </c>
+      <c r="R37" s="4">
+        <v>46101</v>
+      </c>
+      <c r="S37" s="4">
+        <v>46104</v>
+      </c>
+      <c r="T37" s="4">
+        <v>46104</v>
+      </c>
       <c r="V37" s="2" t="s">
         <v>117</v>
       </c>
@@ -4147,7 +4263,7 @@
         <v>29</v>
       </c>
       <c r="X37" s="2" t="s">
-        <v>100</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="1:25" x14ac:dyDescent="0.3">
@@ -4949,6 +5065,9 @@
       <c r="P49" s="4">
         <v>46087</v>
       </c>
+      <c r="T49" s="4">
+        <v>46100</v>
+      </c>
       <c r="V49" s="2" t="s">
         <v>186</v>
       </c>
@@ -5006,6 +5125,9 @@
       <c r="P50" s="4">
         <v>46087</v>
       </c>
+      <c r="T50" s="4">
+        <v>46100</v>
+      </c>
       <c r="V50" s="2" t="s">
         <v>186</v>
       </c>
@@ -5063,6 +5185,9 @@
       <c r="P51" s="4">
         <v>46087</v>
       </c>
+      <c r="T51" s="4">
+        <v>46100</v>
+      </c>
       <c r="V51" s="2" t="s">
         <v>186</v>
       </c>
@@ -5512,6 +5637,9 @@
       <c r="P59" s="4">
         <v>46094</v>
       </c>
+      <c r="Q59" s="4">
+        <v>46103</v>
+      </c>
       <c r="S59" s="4">
         <v>46112</v>
       </c>
@@ -5571,6 +5699,9 @@
       <c r="P60" s="4">
         <v>46094</v>
       </c>
+      <c r="Q60" s="4">
+        <v>46103</v>
+      </c>
       <c r="S60" s="4">
         <v>46112</v>
       </c>
@@ -5630,6 +5761,9 @@
       <c r="P61" s="4">
         <v>46094</v>
       </c>
+      <c r="Q61" s="4">
+        <v>46103</v>
+      </c>
       <c r="S61" s="4">
         <v>46112</v>
       </c>
@@ -5689,6 +5823,9 @@
       <c r="P62" s="4">
         <v>46094</v>
       </c>
+      <c r="Q62" s="4">
+        <v>46103</v>
+      </c>
       <c r="S62" s="4">
         <v>46112</v>
       </c>
@@ -5748,6 +5885,9 @@
       <c r="P63" s="4">
         <v>46094</v>
       </c>
+      <c r="Q63" s="4">
+        <v>46103</v>
+      </c>
       <c r="S63" s="4">
         <v>46112</v>
       </c>
@@ -5807,6 +5947,9 @@
       <c r="P64" s="4">
         <v>46094</v>
       </c>
+      <c r="Q64" s="4">
+        <v>46103</v>
+      </c>
       <c r="S64" s="4">
         <v>46112</v>
       </c>
@@ -5866,6 +6009,9 @@
       <c r="P65" s="4">
         <v>46094</v>
       </c>
+      <c r="Q65" s="4">
+        <v>46103</v>
+      </c>
       <c r="S65" s="4">
         <v>46112</v>
       </c>
@@ -5925,6 +6071,9 @@
       <c r="P66" s="4">
         <v>46094</v>
       </c>
+      <c r="Q66" s="4">
+        <v>46103</v>
+      </c>
       <c r="S66" s="4">
         <v>46112</v>
       </c>
@@ -5984,6 +6133,9 @@
       <c r="P67" s="4">
         <v>46094</v>
       </c>
+      <c r="Q67" s="4">
+        <v>46103</v>
+      </c>
       <c r="S67" s="4">
         <v>46112</v>
       </c>
@@ -6043,6 +6195,9 @@
       <c r="P68" s="4">
         <v>46094</v>
       </c>
+      <c r="Q68" s="4">
+        <v>46103</v>
+      </c>
       <c r="S68" s="4">
         <v>46112</v>
       </c>
@@ -6102,6 +6257,9 @@
       <c r="P69" s="4">
         <v>46094</v>
       </c>
+      <c r="Q69" s="4">
+        <v>46103</v>
+      </c>
       <c r="S69" s="4">
         <v>46112</v>
       </c>
@@ -6161,6 +6319,9 @@
       <c r="P70" s="4">
         <v>46094</v>
       </c>
+      <c r="Q70" s="4">
+        <v>46103</v>
+      </c>
       <c r="S70" s="4">
         <v>46112</v>
       </c>
@@ -6220,6 +6381,9 @@
       <c r="P71" s="4">
         <v>46094</v>
       </c>
+      <c r="Q71" s="4">
+        <v>46103</v>
+      </c>
       <c r="S71" s="4">
         <v>46112</v>
       </c>
@@ -6279,6 +6443,9 @@
       <c r="P72" s="4">
         <v>46094</v>
       </c>
+      <c r="Q72" s="4">
+        <v>46103</v>
+      </c>
       <c r="S72" s="4">
         <v>46112</v>
       </c>
@@ -6324,7 +6491,7 @@
         <v>28</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J73" s="2">
         <v>1</v>
@@ -6337,6 +6504,9 @@
       </c>
       <c r="P73" s="4">
         <v>46094</v>
+      </c>
+      <c r="Q73" s="4">
+        <v>46103</v>
       </c>
       <c r="S73" s="4">
         <v>46112</v>
@@ -6383,7 +6553,7 @@
         <v>28</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="J74" s="2">
         <v>1</v>
@@ -6396,6 +6566,9 @@
       </c>
       <c r="P74" s="4">
         <v>46094</v>
+      </c>
+      <c r="Q74" s="4">
+        <v>46103</v>
       </c>
       <c r="S74" s="4">
         <v>46112</v>
@@ -6456,6 +6629,9 @@
       <c r="P75" s="4">
         <v>46094</v>
       </c>
+      <c r="Q75" s="4">
+        <v>46103</v>
+      </c>
       <c r="S75" s="4">
         <v>46112</v>
       </c>
@@ -6515,6 +6691,9 @@
       <c r="P76" s="4">
         <v>46094</v>
       </c>
+      <c r="Q76" s="4">
+        <v>46103</v>
+      </c>
       <c r="S76" s="4">
         <v>46112</v>
       </c>
@@ -6542,7 +6721,7 @@
         <v>173</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>174</v>
+        <v>45</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>26</v>
@@ -6571,14 +6750,11 @@
       <c r="L77" s="4">
         <v>46086</v>
       </c>
-      <c r="P77" s="4">
-        <v>46094</v>
-      </c>
       <c r="S77" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="T77" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="V77" s="2" t="s">
         <v>149</v>
@@ -6587,7 +6763,7 @@
         <v>30</v>
       </c>
       <c r="X77" s="2" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="Y77" s="2" t="s">
         <v>58</v>
@@ -6601,7 +6777,7 @@
         <v>173</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>174</v>
+        <v>45</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>26</v>
@@ -6630,14 +6806,11 @@
       <c r="L78" s="4">
         <v>46086</v>
       </c>
-      <c r="P78" s="4">
-        <v>46094</v>
-      </c>
       <c r="S78" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="T78" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="V78" s="2" t="s">
         <v>149</v>
@@ -6646,7 +6819,7 @@
         <v>30</v>
       </c>
       <c r="X78" s="2" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="Y78" s="2" t="s">
         <v>58</v>
@@ -6660,7 +6833,7 @@
         <v>173</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>174</v>
+        <v>45</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>26</v>
@@ -6689,14 +6862,11 @@
       <c r="L79" s="4">
         <v>46086</v>
       </c>
-      <c r="P79" s="4">
-        <v>46094</v>
-      </c>
       <c r="S79" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="T79" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="V79" s="2" t="s">
         <v>149</v>
@@ -6705,7 +6875,7 @@
         <v>30</v>
       </c>
       <c r="X79" s="2" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="Y79" s="2" t="s">
         <v>58</v>
@@ -6719,7 +6889,7 @@
         <v>173</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>174</v>
+        <v>45</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>26</v>
@@ -6748,14 +6918,11 @@
       <c r="L80" s="4">
         <v>46086</v>
       </c>
-      <c r="P80" s="4">
-        <v>46094</v>
-      </c>
       <c r="S80" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="T80" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="V80" s="2" t="s">
         <v>149</v>
@@ -6764,7 +6931,7 @@
         <v>30</v>
       </c>
       <c r="X80" s="2" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="Y80" s="2" t="s">
         <v>58</v>
@@ -6778,7 +6945,7 @@
         <v>173</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>174</v>
+        <v>45</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>26</v>
@@ -6807,14 +6974,11 @@
       <c r="L81" s="4">
         <v>46086</v>
       </c>
-      <c r="P81" s="4">
-        <v>46094</v>
-      </c>
       <c r="S81" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="T81" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="V81" s="2" t="s">
         <v>149</v>
@@ -6823,7 +6987,7 @@
         <v>30</v>
       </c>
       <c r="X81" s="2" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="Y81" s="2" t="s">
         <v>58</v>
@@ -6837,7 +7001,7 @@
         <v>173</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>174</v>
+        <v>45</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>26</v>
@@ -6866,14 +7030,11 @@
       <c r="L82" s="4">
         <v>46086</v>
       </c>
-      <c r="P82" s="4">
-        <v>46094</v>
-      </c>
       <c r="S82" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="T82" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="V82" s="2" t="s">
         <v>149</v>
@@ -6882,7 +7043,7 @@
         <v>30</v>
       </c>
       <c r="X82" s="2" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="Y82" s="2" t="s">
         <v>58</v>
@@ -6896,7 +7057,7 @@
         <v>173</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>174</v>
+        <v>45</v>
       </c>
       <c r="D83" s="2" t="s">
         <v>26</v>
@@ -6925,14 +7086,11 @@
       <c r="L83" s="4">
         <v>46086</v>
       </c>
-      <c r="P83" s="4">
-        <v>46094</v>
-      </c>
       <c r="S83" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="T83" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="V83" s="2" t="s">
         <v>149</v>
@@ -6941,7 +7099,7 @@
         <v>30</v>
       </c>
       <c r="X83" s="2" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="Y83" s="2" t="s">
         <v>58</v>
@@ -6955,7 +7113,7 @@
         <v>173</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>174</v>
+        <v>45</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>26</v>
@@ -6984,14 +7142,11 @@
       <c r="L84" s="4">
         <v>46086</v>
       </c>
-      <c r="P84" s="4">
-        <v>46094</v>
-      </c>
       <c r="S84" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="T84" s="4">
-        <v>46112</v>
+        <v>46142</v>
       </c>
       <c r="V84" s="2" t="s">
         <v>149</v>
@@ -7000,7 +7155,7 @@
         <v>30</v>
       </c>
       <c r="X84" s="2" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="Y84" s="2" t="s">
         <v>58</v>
@@ -7008,16 +7163,16 @@
     </row>
     <row r="85" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>153</v>
+        <v>45</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>27</v>
@@ -7026,13 +7181,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G85" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H85" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I85" s="2" t="s">
-        <v>183</v>
+      <c r="I85" s="11" t="s">
+        <v>218</v>
       </c>
       <c r="J85" s="2">
         <v>1</v>
@@ -7041,20 +7196,19 @@
         <v>1</v>
       </c>
       <c r="L85" s="4">
-        <v>46092</v>
-      </c>
-      <c r="M85" s="12"/>
-      <c r="N85" s="4">
-        <v>46093</v>
-      </c>
-      <c r="O85" s="4">
-        <v>46094</v>
+        <v>46086</v>
+      </c>
+      <c r="S85" s="4">
+        <v>46142</v>
+      </c>
+      <c r="T85" s="4">
+        <v>46142</v>
       </c>
       <c r="V85" s="2" t="s">
-        <v>184</v>
+        <v>226</v>
       </c>
       <c r="W85" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X85" s="2" t="s">
         <v>137</v>
@@ -7065,16 +7219,16 @@
     </row>
     <row r="86" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>153</v>
+        <v>45</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>27</v>
@@ -7083,13 +7237,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G86" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H86" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I86" s="2" t="s">
-        <v>176</v>
+      <c r="I86" s="11" t="s">
+        <v>219</v>
       </c>
       <c r="J86" s="2">
         <v>1</v>
@@ -7098,20 +7252,19 @@
         <v>1</v>
       </c>
       <c r="L86" s="4">
-        <v>46092</v>
-      </c>
-      <c r="M86" s="12"/>
-      <c r="N86" s="4">
-        <v>46093</v>
-      </c>
-      <c r="O86" s="4">
-        <v>46094</v>
+        <v>46086</v>
+      </c>
+      <c r="S86" s="4">
+        <v>46142</v>
+      </c>
+      <c r="T86" s="4">
+        <v>46142</v>
       </c>
       <c r="V86" s="2" t="s">
-        <v>184</v>
+        <v>226</v>
       </c>
       <c r="W86" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X86" s="2" t="s">
         <v>137</v>
@@ -7122,16 +7275,16 @@
     </row>
     <row r="87" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>153</v>
+        <v>45</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>27</v>
@@ -7140,13 +7293,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G87" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H87" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I87" s="2" t="s">
-        <v>177</v>
+      <c r="I87" s="11" t="s">
+        <v>220</v>
       </c>
       <c r="J87" s="2">
         <v>1</v>
@@ -7155,20 +7308,19 @@
         <v>1</v>
       </c>
       <c r="L87" s="4">
-        <v>46092</v>
-      </c>
-      <c r="M87" s="12"/>
-      <c r="N87" s="4">
-        <v>46093</v>
-      </c>
-      <c r="O87" s="4">
-        <v>46094</v>
+        <v>46086</v>
+      </c>
+      <c r="S87" s="4">
+        <v>46142</v>
+      </c>
+      <c r="T87" s="4">
+        <v>46142</v>
       </c>
       <c r="V87" s="2" t="s">
-        <v>185</v>
+        <v>226</v>
       </c>
       <c r="W87" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X87" s="2" t="s">
         <v>137</v>
@@ -7179,16 +7331,16 @@
     </row>
     <row r="88" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>153</v>
+        <v>45</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>27</v>
@@ -7197,13 +7349,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G88" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H88" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I88" s="2" t="s">
-        <v>178</v>
+      <c r="I88" s="11" t="s">
+        <v>221</v>
       </c>
       <c r="J88" s="2">
         <v>1</v>
@@ -7212,20 +7364,19 @@
         <v>1</v>
       </c>
       <c r="L88" s="4">
-        <v>46092</v>
-      </c>
-      <c r="M88" s="12"/>
-      <c r="N88" s="4">
-        <v>46093</v>
-      </c>
-      <c r="O88" s="4">
-        <v>46094</v>
+        <v>46086</v>
+      </c>
+      <c r="S88" s="4">
+        <v>46142</v>
+      </c>
+      <c r="T88" s="4">
+        <v>46142</v>
       </c>
       <c r="V88" s="2" t="s">
-        <v>185</v>
+        <v>226</v>
       </c>
       <c r="W88" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X88" s="2" t="s">
         <v>137</v>
@@ -7236,16 +7387,16 @@
     </row>
     <row r="89" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>190</v>
+        <v>45</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>27</v>
@@ -7254,13 +7405,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G89" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H89" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I89" s="2" t="s">
-        <v>191</v>
+      <c r="I89" s="11" t="s">
+        <v>222</v>
       </c>
       <c r="J89" s="2">
         <v>1</v>
@@ -7269,13 +7420,19 @@
         <v>1</v>
       </c>
       <c r="L89" s="4">
-        <v>46094</v>
+        <v>46086</v>
+      </c>
+      <c r="S89" s="4">
+        <v>46142</v>
+      </c>
+      <c r="T89" s="4">
+        <v>46142</v>
       </c>
       <c r="V89" s="2" t="s">
-        <v>184</v>
+        <v>226</v>
       </c>
       <c r="W89" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X89" s="2" t="s">
         <v>137</v>
@@ -7286,16 +7443,16 @@
     </row>
     <row r="90" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>190</v>
+        <v>45</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>27</v>
@@ -7304,13 +7461,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G90" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H90" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I90" s="2" t="s">
-        <v>192</v>
+      <c r="I90" s="11" t="s">
+        <v>223</v>
       </c>
       <c r="J90" s="2">
         <v>1</v>
@@ -7319,13 +7476,19 @@
         <v>1</v>
       </c>
       <c r="L90" s="4">
-        <v>46094</v>
+        <v>46086</v>
+      </c>
+      <c r="S90" s="4">
+        <v>46142</v>
+      </c>
+      <c r="T90" s="4">
+        <v>46142</v>
       </c>
       <c r="V90" s="2" t="s">
-        <v>184</v>
+        <v>226</v>
       </c>
       <c r="W90" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X90" s="2" t="s">
         <v>137</v>
@@ -7336,16 +7499,16 @@
     </row>
     <row r="91" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>190</v>
+        <v>45</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>27</v>
@@ -7354,13 +7517,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G91" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H91" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I91" s="2" t="s">
-        <v>193</v>
+      <c r="I91" s="11" t="s">
+        <v>224</v>
       </c>
       <c r="J91" s="2">
         <v>1</v>
@@ -7369,13 +7532,19 @@
         <v>1</v>
       </c>
       <c r="L91" s="4">
-        <v>46094</v>
+        <v>46086</v>
+      </c>
+      <c r="S91" s="4">
+        <v>46142</v>
+      </c>
+      <c r="T91" s="4">
+        <v>46142</v>
       </c>
       <c r="V91" s="2" t="s">
-        <v>185</v>
+        <v>226</v>
       </c>
       <c r="W91" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X91" s="2" t="s">
         <v>137</v>
@@ -7386,16 +7555,16 @@
     </row>
     <row r="92" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>190</v>
+        <v>45</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>27</v>
@@ -7404,13 +7573,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G92" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H92" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I92" s="2" t="s">
-        <v>195</v>
+      <c r="I92" s="11" t="s">
+        <v>225</v>
       </c>
       <c r="J92" s="2">
         <v>1</v>
@@ -7419,13 +7588,19 @@
         <v>1</v>
       </c>
       <c r="L92" s="4">
-        <v>46094</v>
+        <v>46086</v>
+      </c>
+      <c r="S92" s="4">
+        <v>46142</v>
+      </c>
+      <c r="T92" s="4">
+        <v>46142</v>
       </c>
       <c r="V92" s="2" t="s">
-        <v>185</v>
+        <v>226</v>
       </c>
       <c r="W92" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X92" s="2" t="s">
         <v>137</v>
@@ -7436,16 +7611,16 @@
     </row>
     <row r="93" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>190</v>
+        <v>45</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>27</v>
@@ -7454,13 +7629,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G93" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H93" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I93" s="13" t="s">
-        <v>194</v>
+      <c r="I93" s="11" t="s">
+        <v>227</v>
       </c>
       <c r="J93" s="2">
         <v>1</v>
@@ -7469,13 +7644,19 @@
         <v>1</v>
       </c>
       <c r="L93" s="4">
-        <v>46094</v>
+        <v>46086</v>
+      </c>
+      <c r="S93" s="4">
+        <v>46142</v>
+      </c>
+      <c r="T93" s="4">
+        <v>46142</v>
       </c>
       <c r="V93" s="2" t="s">
-        <v>185</v>
+        <v>226</v>
       </c>
       <c r="W93" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X93" s="2" t="s">
         <v>137</v>
@@ -7486,16 +7667,16 @@
     </row>
     <row r="94" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>190</v>
+        <v>45</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>27</v>
@@ -7504,13 +7685,13 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="G94" s="7">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="H94" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I94" s="2" t="s">
-        <v>196</v>
+      <c r="I94" s="11" t="s">
+        <v>228</v>
       </c>
       <c r="J94" s="2">
         <v>1</v>
@@ -7519,13 +7700,19 @@
         <v>1</v>
       </c>
       <c r="L94" s="4">
-        <v>46098</v>
+        <v>46086</v>
+      </c>
+      <c r="S94" s="4">
+        <v>46142</v>
+      </c>
+      <c r="T94" s="4">
+        <v>46142</v>
       </c>
       <c r="V94" s="2" t="s">
-        <v>199</v>
+        <v>229</v>
       </c>
       <c r="W94" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="X94" s="2" t="s">
         <v>137</v>
@@ -7536,13 +7723,13 @@
     </row>
     <row r="95" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
-        <v>188</v>
+        <v>151</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>189</v>
+        <v>152</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>190</v>
+        <v>153</v>
       </c>
       <c r="D95" s="2" t="s">
         <v>34</v>
@@ -7560,7 +7747,7 @@
         <v>28</v>
       </c>
       <c r="I95" s="2" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="J95" s="2">
         <v>1</v>
@@ -7569,10 +7756,17 @@
         <v>1</v>
       </c>
       <c r="L95" s="4">
-        <v>46098</v>
+        <v>46092</v>
+      </c>
+      <c r="M95" s="12"/>
+      <c r="N95" s="4">
+        <v>46093</v>
+      </c>
+      <c r="O95" s="4">
+        <v>46094</v>
       </c>
       <c r="V95" s="2" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="W95" s="2" t="s">
         <v>29</v>
@@ -7586,13 +7780,13 @@
     </row>
     <row r="96" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
-        <v>188</v>
+        <v>151</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>189</v>
+        <v>152</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>190</v>
+        <v>153</v>
       </c>
       <c r="D96" s="2" t="s">
         <v>34</v>
@@ -7609,8 +7803,8 @@
       <c r="H96" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I96" s="13" t="s">
-        <v>198</v>
+      <c r="I96" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="J96" s="2">
         <v>1</v>
@@ -7619,10 +7813,17 @@
         <v>1</v>
       </c>
       <c r="L96" s="4">
-        <v>46098</v>
+        <v>46092</v>
+      </c>
+      <c r="M96" s="12"/>
+      <c r="N96" s="4">
+        <v>46093</v>
+      </c>
+      <c r="O96" s="4">
+        <v>46094</v>
       </c>
       <c r="V96" s="2" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="W96" s="2" t="s">
         <v>29</v>
@@ -7631,6 +7832,535 @@
         <v>137</v>
       </c>
       <c r="Y96" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="97" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A97" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F97" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G97" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H97" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I97" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="J97" s="2">
+        <v>1</v>
+      </c>
+      <c r="K97" s="2">
+        <v>1</v>
+      </c>
+      <c r="L97" s="4">
+        <v>46092</v>
+      </c>
+      <c r="M97" s="12"/>
+      <c r="N97" s="4">
+        <v>46093</v>
+      </c>
+      <c r="O97" s="4">
+        <v>46094</v>
+      </c>
+      <c r="V97" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="W97" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X97" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="Y97" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="98" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A98" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F98" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G98" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H98" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I98" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="J98" s="2">
+        <v>1</v>
+      </c>
+      <c r="K98" s="2">
+        <v>1</v>
+      </c>
+      <c r="L98" s="4">
+        <v>46092</v>
+      </c>
+      <c r="M98" s="12"/>
+      <c r="N98" s="4">
+        <v>46093</v>
+      </c>
+      <c r="O98" s="4">
+        <v>46094</v>
+      </c>
+      <c r="V98" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="W98" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X98" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="Y98" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="99" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A99" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F99" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G99" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H99" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I99" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="J99" s="2">
+        <v>1</v>
+      </c>
+      <c r="K99" s="2">
+        <v>1</v>
+      </c>
+      <c r="L99" s="4">
+        <v>46094</v>
+      </c>
+      <c r="T99" s="4">
+        <v>46117</v>
+      </c>
+      <c r="V99" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="W99" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X99" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="Y99" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="100" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A100" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F100" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G100" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H100" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I100" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="J100" s="2">
+        <v>1</v>
+      </c>
+      <c r="K100" s="2">
+        <v>1</v>
+      </c>
+      <c r="L100" s="4">
+        <v>46094</v>
+      </c>
+      <c r="T100" s="4">
+        <v>46117</v>
+      </c>
+      <c r="V100" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="W100" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X100" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="Y100" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="101" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A101" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F101" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G101" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H101" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I101" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="J101" s="2">
+        <v>1</v>
+      </c>
+      <c r="K101" s="2">
+        <v>1</v>
+      </c>
+      <c r="L101" s="4">
+        <v>46094</v>
+      </c>
+      <c r="T101" s="4">
+        <v>46117</v>
+      </c>
+      <c r="V101" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="W101" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X101" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="Y101" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="102" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A102" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F102" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G102" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H102" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I102" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="J102" s="2">
+        <v>1</v>
+      </c>
+      <c r="K102" s="2">
+        <v>1</v>
+      </c>
+      <c r="L102" s="4">
+        <v>46094</v>
+      </c>
+      <c r="T102" s="4">
+        <v>46117</v>
+      </c>
+      <c r="V102" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="W102" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X102" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="Y102" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="103" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A103" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F103" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G103" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H103" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I103" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="J103" s="2">
+        <v>1</v>
+      </c>
+      <c r="K103" s="2">
+        <v>1</v>
+      </c>
+      <c r="L103" s="4">
+        <v>46094</v>
+      </c>
+      <c r="T103" s="4">
+        <v>46117</v>
+      </c>
+      <c r="V103" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="W103" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X103" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="Y103" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="104" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A104" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F104" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G104" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H104" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I104" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="J104" s="2">
+        <v>1</v>
+      </c>
+      <c r="K104" s="2">
+        <v>1</v>
+      </c>
+      <c r="L104" s="4">
+        <v>46098</v>
+      </c>
+      <c r="V104" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="W104" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X104" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="Y104" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="105" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A105" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F105" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G105" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H105" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I105" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="J105" s="2">
+        <v>1</v>
+      </c>
+      <c r="K105" s="2">
+        <v>1</v>
+      </c>
+      <c r="L105" s="4">
+        <v>46098</v>
+      </c>
+      <c r="V105" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="W105" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X105" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="Y105" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="106" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A106" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F106" s="3">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G106" s="7">
+        <v>14.5</v>
+      </c>
+      <c r="H106" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I106" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="J106" s="2">
+        <v>1</v>
+      </c>
+      <c r="K106" s="2">
+        <v>1</v>
+      </c>
+      <c r="L106" s="4">
+        <v>46098</v>
+      </c>
+      <c r="V106" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="W106" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X106" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="Y106" s="2" t="s">
         <v>58</v>
       </c>
     </row>
@@ -7638,58 +8368,113 @@
   <autoFilter ref="V1:V42"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="I59:I66">
-    <cfRule type="expression" dxfId="10" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="21" priority="5" stopIfTrue="1">
       <formula>$E3101:$E1048570="sub"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I56:I58">
-    <cfRule type="expression" dxfId="9" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="20" priority="11" stopIfTrue="1">
       <formula>$E3106:$E1048575="sub"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I70">
+    <cfRule type="expression" dxfId="19" priority="72" stopIfTrue="1">
+      <formula>$E6:$E3131="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I83">
+    <cfRule type="expression" dxfId="18" priority="95" stopIfTrue="1">
+      <formula>$E12:$E3136="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I82">
+    <cfRule type="expression" dxfId="17" priority="101" stopIfTrue="1">
+      <formula>$E12:$E3136="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I81">
+    <cfRule type="expression" dxfId="16" priority="107" stopIfTrue="1">
+      <formula>$E12:$E3136="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I80">
-    <cfRule type="expression" dxfId="8" priority="15" stopIfTrue="1">
-      <formula>$E10:$E3124="sub"</formula>
+    <cfRule type="expression" dxfId="15" priority="113" stopIfTrue="1">
+      <formula>$E12:$E3136="sub"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I79">
-    <cfRule type="expression" dxfId="7" priority="19" stopIfTrue="1">
-      <formula>$E10:$E3124="sub"</formula>
+    <cfRule type="expression" dxfId="14" priority="119" stopIfTrue="1">
+      <formula>$E12:$E3136="sub"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I78">
-    <cfRule type="expression" dxfId="6" priority="23" stopIfTrue="1">
-      <formula>$E10:$E3124="sub"</formula>
+    <cfRule type="expression" dxfId="13" priority="125" stopIfTrue="1">
+      <formula>$E12:$E3136="sub"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I84">
-    <cfRule type="expression" dxfId="5" priority="45" stopIfTrue="1">
-      <formula>$E11:$E3125="sub"</formula>
+  <conditionalFormatting sqref="I90">
+    <cfRule type="expression" dxfId="12" priority="149" stopIfTrue="1">
+      <formula>$E13:$E3137="sub"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I83">
-    <cfRule type="expression" dxfId="4" priority="50" stopIfTrue="1">
-      <formula>$E11:$E3125="sub"</formula>
+  <conditionalFormatting sqref="I89">
+    <cfRule type="expression" dxfId="11" priority="156" stopIfTrue="1">
+      <formula>$E13:$E3137="sub"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I81:I82">
-    <cfRule type="expression" dxfId="3" priority="54" stopIfTrue="1">
-      <formula>$E10:$E3124="sub"</formula>
+  <conditionalFormatting sqref="I88">
+    <cfRule type="expression" dxfId="10" priority="163" stopIfTrue="1">
+      <formula>$E13:$E3137="sub"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I76:I77">
-    <cfRule type="expression" dxfId="2" priority="55" stopIfTrue="1">
-      <formula>$E9:$E3123="sub"</formula>
+  <conditionalFormatting sqref="I87">
+    <cfRule type="expression" dxfId="9" priority="170" stopIfTrue="1">
+      <formula>$E13:$E3137="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I86">
+    <cfRule type="expression" dxfId="8" priority="177" stopIfTrue="1">
+      <formula>$E13:$E3137="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I94">
+    <cfRule type="expression" dxfId="7" priority="213" stopIfTrue="1">
+      <formula>$E15:$E3139="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I91:I93">
+    <cfRule type="expression" dxfId="6" priority="220" stopIfTrue="1">
+      <formula>$E13:$E3137="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I84:I85">
+    <cfRule type="expression" dxfId="5" priority="221" stopIfTrue="1">
+      <formula>$E12:$E3136="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I73:I74">
+    <cfRule type="expression" dxfId="4" priority="222" stopIfTrue="1">
+      <formula>$E9:$E3133="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I68:I69">
+    <cfRule type="expression" dxfId="3" priority="223" stopIfTrue="1">
+      <formula>$E2:$E3127="sub"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I75:I77">
+    <cfRule type="expression" dxfId="2" priority="224" stopIfTrue="1">
+      <formula>$E10:$E3134="sub"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I67">
-    <cfRule type="expression" dxfId="1" priority="56" stopIfTrue="1">
-      <formula>$E3115:$E1048576="sub"</formula>
+    <cfRule type="expression" dxfId="1" priority="225" stopIfTrue="1">
+      <formula>$E3125:$E1048576="sub"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I68:I75">
-    <cfRule type="expression" dxfId="0" priority="57" stopIfTrue="1">
-      <formula>$E2:$E3117="sub"</formula>
+  <conditionalFormatting sqref="I71:I72">
+    <cfRule type="expression" dxfId="0" priority="226" stopIfTrue="1">
+      <formula>$E8:$E3133="sub"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>